<commit_message>
Enhance Apps Script with dynamic dropdown inheritance and comprehensive source channel list to prevent invalid warnings
</commit_message>
<xml_diff>
--- a/KTA_Executive_Marketing_CRM_Tracker.xlsx
+++ b/KTA_Executive_Marketing_CRM_Tracker.xlsx
@@ -790,7 +790,7 @@
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
@@ -6402,7 +6402,7 @@
   </conditionalFormatting>
   <dataValidations count="5">
     <dataValidation sqref="D7:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Website RFQ,AI Chatbot,Chef Sample Box,WhatsApp Desk,Inbound Call,Wholesale Portal"</formula1>
+      <formula1>"Website RFQ,AI Chatbot,Chef Sample Box,Corporate Partnership Registration,General Trade Desk Inquiry,Chef Dispatches Newsletter,WhatsApp Desk,Wholesale Portal,Inbound Call"</formula1>
     </dataValidation>
     <dataValidation sqref="M7:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Anand R. (Trade Desk),Kavitha S. (Hospitality),Suresh M. (Wholesale),Praveen K. (Key Accounts)"</formula1>
@@ -6427,7 +6427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6725,19 +6725,19 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>WhatsApp Desk</t>
+          <t>Corporate Partnership</t>
         </is>
       </c>
       <c r="B17" s="33">
-        <f>COUNTIF('Inbound Leads'!D7:D1000, "WhatsApp Desk")</f>
+        <f>COUNTIF('Inbound Leads'!D7:D1000, "*Partnership*")</f>
         <v/>
       </c>
       <c r="C17" s="33">
-        <f>COUNTIFS('Inbound Leads'!D7:D1000, "WhatsApp Desk", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <f>COUNTIFS('Inbound Leads'!D7:D1000, "*Partnership*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "WhatsApp Desk", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "*Partnership*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
         <v/>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -6757,19 +6757,19 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>Wholesale Portal</t>
+          <t>General Trade Desk</t>
         </is>
       </c>
       <c r="B18" s="31">
-        <f>COUNTIF('Inbound Leads'!D7:D1000, "Wholesale Portal")</f>
+        <f>COUNTIF('Inbound Leads'!D7:D1000, "*Trade Desk*")</f>
         <v/>
       </c>
       <c r="C18" s="31">
-        <f>COUNTIFS('Inbound Leads'!D7:D1000, "Wholesale Portal", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <f>COUNTIFS('Inbound Leads'!D7:D1000, "*Trade Desk*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
         <v/>
       </c>
       <c r="D18" s="32">
-        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "Wholesale Portal", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "*Trade Desk*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
         <v/>
       </c>
       <c r="F18" s="34" t="inlineStr">
@@ -6789,38 +6789,95 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
+          <t>Chef Newsletter</t>
+        </is>
+      </c>
+      <c r="B19" s="33">
+        <f>COUNTIF('Inbound Leads'!D7:D1000, "*Newsletter*")</f>
+        <v/>
+      </c>
+      <c r="C19" s="33">
+        <f>COUNTIFS('Inbound Leads'!D7:D1000, "*Newsletter*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <v/>
+      </c>
+      <c r="D19" s="16">
+        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "*Newsletter*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>WhatsApp Desk</t>
+        </is>
+      </c>
+      <c r="B20" s="31">
+        <f>COUNTIF('Inbound Leads'!D7:D1000, "*WhatsApp*")</f>
+        <v/>
+      </c>
+      <c r="C20" s="31">
+        <f>COUNTIFS('Inbound Leads'!D7:D1000, "*WhatsApp*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <v/>
+      </c>
+      <c r="D20" s="32">
+        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "*WhatsApp*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Wholesale Portal</t>
+        </is>
+      </c>
+      <c r="B21" s="33">
+        <f>COUNTIF('Inbound Leads'!D7:D1000, "*Wholesale*")</f>
+        <v/>
+      </c>
+      <c r="C21" s="33">
+        <f>COUNTIFS('Inbound Leads'!D7:D1000, "*Wholesale*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <v/>
+      </c>
+      <c r="D21" s="16">
+        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "*Wholesale*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
           <t>Inbound Call</t>
         </is>
       </c>
-      <c r="B19" s="33">
-        <f>COUNTIF('Inbound Leads'!D7:D1000, "Inbound Call")</f>
+      <c r="B22" s="31">
+        <f>COUNTIF('Inbound Leads'!D7:D1000, "*Call*")</f>
         <v/>
       </c>
-      <c r="C19" s="33">
-        <f>COUNTIFS('Inbound Leads'!D7:D1000, "Inbound Call", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+      <c r="C22" s="31">
+        <f>COUNTIFS('Inbound Leads'!D7:D1000, "*Call*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
         <v/>
       </c>
-      <c r="D19" s="16">
-        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "Inbound Call", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
+      <c r="D22" s="32">
+        <f>SUMIFS('Inbound Leads'!Q7:Q1000, 'Inbound Leads'!D7:D1000, "*Call*", 'Inbound Leads'!O7:O1000, "Closed Won")</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="34" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="34" t="inlineStr">
         <is>
           <t>TOTAL INBOUND</t>
         </is>
       </c>
-      <c r="B20" s="35">
-        <f>SUM(B14:B19)</f>
+      <c r="B23" s="35">
+        <f>SUM(B14:B22)</f>
         <v/>
       </c>
-      <c r="C20" s="35">
-        <f>SUM(C14:C19)</f>
+      <c r="C23" s="35">
+        <f>SUM(C14:C22)</f>
         <v/>
       </c>
-      <c r="D20" s="36">
-        <f>SUM(D14:D19)</f>
+      <c r="D23" s="36">
+        <f>SUM(D14:D22)</f>
         <v/>
       </c>
     </row>

</xml_diff>